<commit_message>
Update generated output after column_mapping_v2.csv fix
Regenerated by running main.py after fixing the section-12 column
name mapping.
</commit_message>
<xml_diff>
--- a/output/нужна_проверка.xlsx
+++ b/output/нужна_проверка.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,69 +460,69 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t29Ved14.xlsx</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
         <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>коммерческие и управленческие расходы</t>
+          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.73</v>
+        <v>0.57</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>в том числе управленческие расходы</t>
+          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DohIRasPoObyVidDeyZaOtcPerVToChiUprRas_1</t>
+          <t>PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>64</v>
+        <v>127</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>T24_000000_t23Ved14mo8.xlsx</t>
+          <t>T24_000000_t29Ved14.xlsx</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>себестоимость продаж с учетом коммерческих и управленческих расходов</t>
+          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.53</v>
+        <v>0.57</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>в том числе управленческие расходы</t>
+          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DohIRasPoObyVidDeyZaOtcPerVToChiUprRas_1</t>
+          <t>PlPoFin3</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
         <v>3</v>
@@ -589,74 +589,6 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
-        <is>
-          <t>PlPoFin3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>127</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>T24_000000_t29Ved14.xlsx</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>PlPoFin3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>127</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>T24_000000_t29Ved14.xlsx</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>14</v>
-      </c>
-      <c r="D7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>PlPoFin3</t>
         </is>

</xml_diff>

<commit_message>
Auto-tolerate group-header prefixes shared by sibling indicators
column_mapping_v2.csv often inherits a merged multi-column group
header from Excel (e.g. "Отчетный год Прочее"), which Word doesn't
repeat per column. generate_word_template now detects prefixes that
are genuinely shared by 2+ indicators of the same source file and
retries matching with that prefix stripped, instead of relying only
on the CSV being hand-curated per file. Logged to a new optional
group_prefix_match_report_path for review.
</commit_message>
<xml_diff>
--- a/output/нужна_проверка.xlsx
+++ b/output/нужна_проверка.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -468,33 +468,33 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
         <v>3</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
+          <t>в том числе прочие поступления</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
+          <t>поступления по текущей деятельности прочие поступления</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PlPoFin3</t>
+          <t>PrTekDeVsego</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -502,33 +502,33 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
         <v>3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
+          <t>в том числе прочие поступления</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
+          <t>поступления по текущей деятельности прочие поступления</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>PlPoFin3</t>
+          <t>PrTekDeVsego</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -536,61 +536,741 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
         <v>3</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
+          <t>в том числе прочие поступления</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
+          <t>поступления по текущей деятельности прочие поступления</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PlPoFin3</t>
+          <t>PrTekDeVsego</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
+        <v>109</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>110</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>111</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>112</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>112</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>117</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>117</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>118</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>119</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>120</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>120</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" t="n">
+        <v>13</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>в том числе прочие поступления</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>поступления по текущей деятельности прочие поступления</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>PrTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
         <v>127</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>T24_000000_t29Ved14.xlsx</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>11</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>PlPoFin3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>127</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>PlPoFin3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>127</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>13</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>PlPoFin3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>127</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>14</v>
       </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>продолжение таблицы 20 в том числе от выпуска облигаций векселей и других долговых ценных бумаг и др</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F19" t="n">
         <v>0.57</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>в связи с погашением выкупом векселей и других долговых ценных бумаг возврат кредитов и займов</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>PlPoFin3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>132</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>платежи всего</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>платежи по текущей деятельности всего</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>PlatPoTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>132</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>платежи всего</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>платежи по текущей деятельности всего</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>PlatPoTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>132</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>9</v>
+      </c>
+      <c r="D22" t="n">
+        <v>18</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>платежи всего</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>платежи по текущей деятельности всего</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>PlatPoTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>132</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" t="n">
+        <v>18</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>платежи всего</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>платежи по текущей деятельности всего</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>PlatPoTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>132</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>9</v>
+      </c>
+      <c r="D24" t="n">
+        <v>33</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>платежи всего</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>платежи по текущей деятельности всего</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>PlatPoTekDeVsego</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>132</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>T24_000000_t29Ved14.xlsx</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" t="n">
+        <v>33</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>платежи всего</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>платежи по текущей деятельности всего</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>PlatPoTekDeVsego</t>
         </is>
       </c>
     </row>

</xml_diff>